<commit_message>
daily sale till 20
</commit_message>
<xml_diff>
--- a/Aug_2026/Daily Sales/20-08-26/Furqan.xlsx
+++ b/Aug_2026/Daily Sales/20-08-26/Furqan.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29127"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BCE8362-19C1-49E3-9D49-62757DC48BFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C87A90DA-2EE6-4B40-B1CC-0E6CAAB70B52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="594" firstSheet="3" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" tabRatio="594" firstSheet="3" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Dist Price List (2)" sheetId="41" state="hidden" r:id="rId1"/>
@@ -55,7 +55,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3978" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3978" uniqueCount="534">
   <si>
     <t>Sr.No</t>
   </si>
@@ -1654,6 +1654,9 @@
   </si>
   <si>
     <t>Address: Guru mangat</t>
+  </si>
+  <si>
+    <t>NTN  #: 6110128821443</t>
   </si>
 </sst>
 </file>
@@ -12963,7 +12966,7 @@
     </row>
     <row r="7" spans="1:22 16383:16384" s="87" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A7" s="392" t="s">
-        <v>73</v>
+        <v>533</v>
       </c>
       <c r="B7" s="392"/>
       <c r="C7" s="392"/>
@@ -13325,20 +13328,18 @@
         <v>52.462499999999999</v>
       </c>
       <c r="G17" s="287"/>
-      <c r="H17" s="96">
-        <v>10</v>
-      </c>
+      <c r="H17" s="96"/>
       <c r="I17" s="236">
         <f t="shared" ref="I17:I23" si="0">(G17*D17)*F17+H17*F17</f>
-        <v>524.625</v>
+        <v>0</v>
       </c>
       <c r="J17" s="272">
         <f t="shared" ref="J17:L24" si="1">$I17*S17</f>
-        <v>41.97</v>
+        <v>0</v>
       </c>
       <c r="K17" s="128">
         <f>$I17*T17</f>
-        <v>18.361875000000001</v>
+        <v>0</v>
       </c>
       <c r="L17" s="119">
         <f>$I17*U17</f>
@@ -13346,19 +13347,19 @@
       </c>
       <c r="M17" s="230">
         <f t="shared" ref="M17:M24" si="2">I17-SUM(J17:L17)</f>
-        <v>464.29312500000003</v>
+        <v>0</v>
       </c>
       <c r="N17" s="277">
         <f t="shared" ref="N17:N24" si="3">+(G17*D17+H17)*V17</f>
-        <v>99.152542372881314</v>
+        <v>0</v>
       </c>
       <c r="O17" s="239">
         <f t="shared" ref="O17:O24" si="4">(N17+M17)*$O$15</f>
-        <v>2.8172283368644067</v>
+        <v>0</v>
       </c>
       <c r="P17" s="311">
         <f t="shared" ref="P17:P24" si="5">M17+N17+O17</f>
-        <v>566.26289570974575</v>
+        <v>0</v>
       </c>
       <c r="Q17" s="156"/>
       <c r="S17" s="269">
@@ -13476,18 +13477,20 @@
         <v>72.64</v>
       </c>
       <c r="G19" s="287"/>
-      <c r="H19" s="96"/>
+      <c r="H19" s="96">
+        <v>10</v>
+      </c>
       <c r="I19" s="236">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>726.4</v>
       </c>
       <c r="J19" s="272">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>58.112000000000002</v>
       </c>
       <c r="K19" s="128">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>25.424000000000003</v>
       </c>
       <c r="L19" s="119">
         <f t="shared" si="1"/>
@@ -13495,19 +13498,19 @@
       </c>
       <c r="M19" s="230">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>642.86400000000003</v>
       </c>
       <c r="N19" s="277">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>137.28813559322035</v>
       </c>
       <c r="O19" s="239">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>3.9007606779661019</v>
       </c>
       <c r="P19" s="311">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>784.05289627118646</v>
       </c>
       <c r="Q19" s="156"/>
       <c r="S19" s="269">
@@ -13627,18 +13630,20 @@
         <v>72.64</v>
       </c>
       <c r="G21" s="287"/>
-      <c r="H21" s="96"/>
+      <c r="H21" s="96">
+        <v>20</v>
+      </c>
       <c r="I21" s="236">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1452.8</v>
       </c>
       <c r="J21" s="272">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>116.224</v>
       </c>
       <c r="K21" s="128">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>50.848000000000006</v>
       </c>
       <c r="L21" s="119">
         <f t="shared" si="1"/>
@@ -13646,19 +13651,19 @@
       </c>
       <c r="M21" s="230">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1285.7280000000001</v>
       </c>
       <c r="N21" s="277">
         <f t="shared" si="3"/>
-        <v>0</v>
+        <v>274.57627118644069</v>
       </c>
       <c r="O21" s="239">
         <f t="shared" si="4"/>
-        <v>0</v>
+        <v>7.8015213559322039</v>
       </c>
       <c r="P21" s="311">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>1568.1057925423729</v>
       </c>
       <c r="Q21" s="156"/>
       <c r="S21" s="269">
@@ -13700,40 +13705,38 @@
         <v>39.230000000000004</v>
       </c>
       <c r="G22" s="287"/>
-      <c r="H22" s="96">
-        <v>20</v>
-      </c>
+      <c r="H22" s="96"/>
       <c r="I22" s="236">
         <f t="shared" si="0"/>
-        <v>784.60000000000014</v>
+        <v>0</v>
       </c>
       <c r="J22" s="272">
         <f t="shared" si="1"/>
-        <v>39.230000000000011</v>
+        <v>0</v>
       </c>
       <c r="K22" s="128">
         <f t="shared" si="1"/>
-        <v>27.461000000000006</v>
+        <v>0</v>
       </c>
       <c r="L22" s="119">
         <f t="shared" si="1"/>
-        <v>40.014600000000002</v>
+        <v>0</v>
       </c>
       <c r="M22" s="230">
         <f t="shared" si="2"/>
-        <v>677.89440000000013</v>
+        <v>0</v>
       </c>
       <c r="N22" s="277">
         <f t="shared" si="3"/>
-        <v>152.54237288135585</v>
+        <v>0</v>
       </c>
       <c r="O22" s="239">
         <f t="shared" si="4"/>
-        <v>4.1521838644067799</v>
+        <v>0</v>
       </c>
       <c r="P22" s="311">
         <f t="shared" si="5"/>
-        <v>834.58895674576274</v>
+        <v>0</v>
       </c>
       <c r="Q22" s="156"/>
       <c r="S22" s="269">
@@ -13922,35 +13925,35 @@
       </c>
       <c r="I25" s="114">
         <f t="shared" si="7"/>
-        <v>2035.6250000000002</v>
+        <v>2905.6</v>
       </c>
       <c r="J25" s="274">
         <f>SUM(J16:J24)</f>
-        <v>139.31200000000001</v>
+        <v>232.44800000000001</v>
       </c>
       <c r="K25" s="275">
         <f t="shared" si="7"/>
-        <v>71.246875000000017</v>
+        <v>101.69600000000001</v>
       </c>
       <c r="L25" s="276">
         <f t="shared" si="7"/>
-        <v>40.014600000000002</v>
+        <v>0</v>
       </c>
       <c r="M25" s="232">
         <f t="shared" si="7"/>
-        <v>1785.0515250000003</v>
+        <v>2571.4560000000001</v>
       </c>
       <c r="N25" s="233">
         <f>SUM(N16:N24)</f>
-        <v>388.98305084745749</v>
+        <v>549.15254237288138</v>
       </c>
       <c r="O25" s="101">
         <f>SUM(O16:O24)</f>
-        <v>10.870172879237288</v>
+        <v>15.603042711864408</v>
       </c>
       <c r="P25" s="113">
         <f>SUM(P16:P24)</f>
-        <v>2184.9047487266953</v>
+        <v>3136.2115850847458</v>
       </c>
       <c r="Q25" s="128">
         <f>SUM(Q16:Q24)</f>
@@ -14004,7 +14007,7 @@
       <c r="O28" s="366"/>
       <c r="P28" s="139">
         <f>I25</f>
-        <v>2035.6250000000002</v>
+        <v>2905.6</v>
       </c>
     </row>
     <row r="29" spans="1:22 16384:16384" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -14025,7 +14028,7 @@
       <c r="O29" s="368"/>
       <c r="P29" s="140">
         <f>+J25</f>
-        <v>139.31200000000001</v>
+        <v>232.44800000000001</v>
       </c>
     </row>
     <row r="30" spans="1:22 16384:16384" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -14046,7 +14049,7 @@
       <c r="O30" s="368"/>
       <c r="P30" s="140">
         <f>+K25+L25</f>
-        <v>111.26147500000002</v>
+        <v>101.69600000000001</v>
       </c>
     </row>
     <row r="31" spans="1:22 16384:16384" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -14068,7 +14071,7 @@
       <c r="O31" s="368"/>
       <c r="P31" s="140">
         <f>P28-P29-P30</f>
-        <v>1785.0515250000001</v>
+        <v>2571.4560000000001</v>
       </c>
     </row>
     <row r="32" spans="1:22 16384:16384" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -14092,7 +14095,7 @@
       </c>
       <c r="P32" s="140">
         <f>+N25</f>
-        <v>388.98305084745749</v>
+        <v>549.15254237288138</v>
       </c>
     </row>
     <row r="33" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -14114,7 +14117,7 @@
       <c r="O33" s="370"/>
       <c r="P33" s="140">
         <f>P31+P32</f>
-        <v>2174.0345758474577</v>
+        <v>3120.6085423728814</v>
       </c>
     </row>
     <row r="34" spans="2:16" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -14139,7 +14142,7 @@
       </c>
       <c r="P34" s="140">
         <f>O34*P33</f>
-        <v>10.870172879237289</v>
+        <v>15.603042711864408</v>
       </c>
     </row>
     <row r="35" spans="2:16" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
@@ -14149,7 +14152,7 @@
       <c r="O35" s="372"/>
       <c r="P35" s="297">
         <f>+P33+P34</f>
-        <v>2184.9047487266948</v>
+        <v>3136.2115850847458</v>
       </c>
     </row>
     <row r="36" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
@@ -47950,7 +47953,7 @@
       <c r="L4" s="392"/>
       <c r="M4" s="395">
         <f ca="1">TODAY()+1</f>
-        <v>46254</v>
+        <v>46255</v>
       </c>
       <c r="N4" s="395"/>
       <c r="O4" s="395"/>
@@ -47978,7 +47981,7 @@
       <c r="L5" s="392"/>
       <c r="M5" s="395">
         <f ca="1">M4-1</f>
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="N5" s="391"/>
       <c r="O5" s="391"/>
@@ -54176,7 +54179,7 @@
       <c r="G3" s="387"/>
       <c r="H3" s="384">
         <f ca="1">TODAY()</f>
-        <v>46253</v>
+        <v>46254</v>
       </c>
       <c r="I3" s="384"/>
       <c r="J3" s="385"/>
@@ -54451,19 +54454,19 @@
       </c>
       <c r="H8" s="309">
         <f>+'1'!H17+'2'!H17+'3'!H17+'4'!H17+'5'!H17+'6'!H17+'7'!H17+'8'!H17+'9'!H17+'10'!H17+'11'!H17+'12'!H17+'13'!H17+'14'!H17+'15'!H17+'16'!H17+'17'!H17+'18'!H17+'19'!H17+'20'!H17+'21'!H17+'22'!H17+'23'!H17+'24'!H17+'25'!H17+'26'!H17+'27'!H17+'28'!H17+'29'!H17+'30'!H17</f>
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="I8" s="236">
         <f t="shared" ref="I8:I14" si="0">(G8*D8)*F8+H8*F8</f>
-        <v>2832.9749999999999</v>
+        <v>2308.35</v>
       </c>
       <c r="J8" s="286">
         <f>+'1'!J17+'2'!J17+'3'!J17+'4'!J17+'5'!J17+'6'!J17+'7'!J17+'8'!J17+'9'!J17+'10'!J17+'11'!J17+'12'!J17+'13'!J17+'14'!J17+'15'!J17+'16'!J17+'17'!J17+'18'!J17+'19'!J17+'20'!J17+'21'!J17+'22'!J17+'23'!J17+'24'!J17+'25'!J17+'26'!J17+'27'!J17+'28'!J17+'29'!J17+'30'!J17</f>
-        <v>226.63800000000001</v>
+        <v>184.66800000000001</v>
       </c>
       <c r="K8" s="286">
         <f>+'1'!K17+'2'!K17+'3'!K17+'4'!K17+'5'!K17+'6'!K17+'7'!K17+'8'!K17+'9'!K17+'10'!K17+'11'!K17+'12'!K17+'13'!K17+'14'!K17+'15'!K17+'16'!K17+'17'!K17+'18'!K17+'19'!K17+'20'!K17+'21'!K17+'22'!K17+'23'!K17+'24'!K17+'25'!K17+'26'!K17+'27'!K17+'28'!K17+'29'!K17+'30'!K17</f>
-        <v>99.154124999999993</v>
+        <v>80.792249999999996</v>
       </c>
       <c r="L8" s="286">
         <f>+'1'!L17+'2'!L17+'3'!L17+'4'!L17+'5'!L17+'6'!L17+'7'!L17+'8'!L17+'9'!L17+'10'!L17+'11'!L17+'12'!L17+'13'!L17+'14'!L17+'15'!L17+'16'!L17+'17'!L17+'18'!L17+'19'!L17+'20'!L17+'21'!L17+'22'!L17+'23'!L17+'24'!L17+'25'!L17+'26'!L17+'27'!L17+'28'!L17+'29'!L17+'30'!L17</f>
@@ -54471,19 +54474,19 @@
       </c>
       <c r="M8" s="230">
         <f t="shared" ref="M8:M15" si="1">I8-SUM(J8:L8)</f>
-        <v>2507.182875</v>
+        <v>2042.8897499999998</v>
       </c>
       <c r="N8" s="286">
         <f>+'1'!N17+'2'!N17+'3'!N17+'4'!N17+'5'!N17+'6'!N17+'7'!N17+'8'!N17+'9'!N17+'10'!N17+'11'!N17+'12'!N17+'13'!N17+'14'!N17+'15'!N17+'16'!N17+'17'!N17+'18'!N17+'19'!N17+'20'!N17+'21'!N17+'22'!N17+'23'!N17+'24'!N17+'25'!N17+'26'!N17+'27'!N17+'28'!N17+'29'!N17+'30'!N17</f>
-        <v>535.42372881355902</v>
+        <v>436.27118644067775</v>
       </c>
       <c r="O8" s="286">
         <f>+'1'!O17+'2'!O17+'3'!O17+'4'!O17+'5'!O17+'6'!O17+'7'!O17+'8'!O17+'9'!O17+'10'!O17+'11'!O17+'12'!O17+'13'!O17+'14'!O17+'15'!O17+'16'!O17+'17'!O17+'18'!O17+'19'!O17+'20'!O17+'21'!O17+'22'!O17+'23'!O17+'24'!O17+'25'!O17+'26'!O17+'27'!O17+'28'!O17+'29'!O17+'30'!O17</f>
-        <v>15.213033019067797</v>
+        <v>12.395804682203391</v>
       </c>
       <c r="P8" s="311">
         <f t="shared" ref="P8:P15" si="2">M8+N8+O8</f>
-        <v>3057.8196368326271</v>
+        <v>2491.5567411228812</v>
       </c>
       <c r="Q8" s="213">
         <f>+'1'!Q17+'2'!Q17+'3'!Q17+'4'!Q17+'5'!Q17+'6'!Q17+'7'!Q17+'8'!Q17+'9'!Q17+'10'!Q17+'11'!Q17+'12'!Q17+'13'!Q17+'14'!Q17+'15'!Q17+'16'!Q17+'17'!Q17+'18'!Q17+'19'!Q17+'20'!Q17+'21'!Q17+'22'!Q17+'23'!Q17+'24'!Q17+'25'!Q17+'26'!Q17+'27'!Q17+'28'!Q17+'29'!Q17+'30'!Q17</f>
@@ -54614,19 +54617,19 @@
       </c>
       <c r="H10" s="309">
         <f>+'1'!H19+'2'!H19+'3'!H19+'4'!H19+'5'!H19+'6'!H19+'7'!H19+'8'!H19+'9'!H19+'10'!H19+'11'!H19+'12'!H19+'13'!H19+'14'!H19+'15'!H19+'16'!H19+'17'!H19+'18'!H19+'19'!H19+'20'!H19+'21'!H19+'22'!H19+'23'!H19+'24'!H19+'25'!H19+'26'!H19+'27'!H19+'28'!H19+'29'!H19+'30'!H19</f>
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="I10" s="236">
         <f t="shared" si="0"/>
-        <v>2251.84</v>
+        <v>2978.2400000000002</v>
       </c>
       <c r="J10" s="286">
         <f>+'1'!J19+'2'!J19+'3'!J19+'4'!J19+'5'!J19+'6'!J19+'7'!J19+'8'!J19+'9'!J19+'10'!J19+'11'!J19+'12'!J19+'13'!J19+'14'!J19+'15'!J19+'16'!J19+'17'!J19+'18'!J19+'19'!J19+'20'!J19+'21'!J19+'22'!J19+'23'!J19+'24'!J19+'25'!J19+'26'!J19+'27'!J19+'28'!J19+'29'!J19+'30'!J19</f>
-        <v>180.14720000000003</v>
+        <v>238.25920000000002</v>
       </c>
       <c r="K10" s="286">
         <f>+'1'!K19+'2'!K19+'3'!K19+'4'!K19+'5'!K19+'6'!K19+'7'!K19+'8'!K19+'9'!K19+'10'!K19+'11'!K19+'12'!K19+'13'!K19+'14'!K19+'15'!K19+'16'!K19+'17'!K19+'18'!K19+'19'!K19+'20'!K19+'21'!K19+'22'!K19+'23'!K19+'24'!K19+'25'!K19+'26'!K19+'27'!K19+'28'!K19+'29'!K19+'30'!K19</f>
-        <v>78.814400000000006</v>
+        <v>104.23840000000001</v>
       </c>
       <c r="L10" s="286">
         <f>+'1'!L19+'2'!L19+'3'!L19+'4'!L19+'5'!L19+'6'!L19+'7'!L19+'8'!L19+'9'!L19+'10'!L19+'11'!L19+'12'!L19+'13'!L19+'14'!L19+'15'!L19+'16'!L19+'17'!L19+'18'!L19+'19'!L19+'20'!L19+'21'!L19+'22'!L19+'23'!L19+'24'!L19+'25'!L19+'26'!L19+'27'!L19+'28'!L19+'29'!L19+'30'!L19</f>
@@ -54634,19 +54637,19 @@
       </c>
       <c r="M10" s="230">
         <f t="shared" si="1"/>
-        <v>1992.8784000000001</v>
+        <v>2635.7424000000001</v>
       </c>
       <c r="N10" s="286">
         <f>+'1'!N19+'2'!N19+'3'!N19+'4'!N19+'5'!N19+'6'!N19+'7'!N19+'8'!N19+'9'!N19+'10'!N19+'11'!N19+'12'!N19+'13'!N19+'14'!N19+'15'!N19+'16'!N19+'17'!N19+'18'!N19+'19'!N19+'20'!N19+'21'!N19+'22'!N19+'23'!N19+'24'!N19+'25'!N19+'26'!N19+'27'!N19+'28'!N19+'29'!N19+'30'!N19</f>
-        <v>425.59322033898309</v>
+        <v>562.88135593220341</v>
       </c>
       <c r="O10" s="286">
         <f>+'1'!O19+'2'!O19+'3'!O19+'4'!O19+'5'!O19+'6'!O19+'7'!O19+'8'!O19+'9'!O19+'10'!O19+'11'!O19+'12'!O19+'13'!O19+'14'!O19+'15'!O19+'16'!O19+'17'!O19+'18'!O19+'19'!O19+'20'!O19+'21'!O19+'22'!O19+'23'!O19+'24'!O19+'25'!O19+'26'!O19+'27'!O19+'28'!O19+'29'!O19+'30'!O19</f>
-        <v>12.092358101694916</v>
+        <v>15.993118779661017</v>
       </c>
       <c r="P10" s="311">
         <f t="shared" si="2"/>
-        <v>2430.5639784406781</v>
+        <v>3214.6168747118645</v>
       </c>
       <c r="Q10" s="213">
         <f>+'1'!Q19+'2'!Q19+'3'!Q19+'4'!Q19+'5'!Q19+'6'!Q19+'7'!Q19+'8'!Q19+'9'!Q19+'10'!Q19+'11'!Q19+'12'!Q19+'13'!Q19+'14'!Q19+'15'!Q19+'16'!Q19+'17'!Q19+'18'!Q19+'19'!Q19+'20'!Q19+'21'!Q19+'22'!Q19+'23'!Q19+'24'!Q19+'25'!Q19+'26'!Q19+'27'!Q19+'28'!Q19+'29'!Q19+'30'!Q19</f>
@@ -54774,19 +54777,19 @@
       </c>
       <c r="H12" s="309">
         <f>+'1'!H21+'2'!H21+'3'!H21+'4'!H21+'5'!H21+'6'!H21+'7'!H21+'8'!H21+'9'!H21+'10'!H21+'11'!H21+'12'!H21+'13'!H21+'14'!H21+'15'!H21+'16'!H21+'17'!H21+'18'!H21+'19'!H21+'20'!H21+'21'!H21+'22'!H21+'23'!H21+'24'!H21+'25'!H21+'26'!H21+'27'!H21+'28'!H21+'29'!H21+'30'!H21</f>
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I12" s="236">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1452.8</v>
       </c>
       <c r="J12" s="286">
         <f>+'1'!J21+'2'!J21+'3'!J21+'4'!J21+'5'!J21+'6'!J21+'7'!J21+'8'!J21+'9'!J21+'10'!J21+'11'!J21+'12'!J21+'13'!J21+'14'!J21+'15'!J21+'16'!J21+'17'!J21+'18'!J21+'19'!J21+'20'!J21+'21'!J21+'22'!J21+'23'!J21+'24'!J21+'25'!J21+'26'!J21+'27'!J21+'28'!J21+'29'!J21+'30'!J21</f>
-        <v>0</v>
+        <v>116.224</v>
       </c>
       <c r="K12" s="286">
         <f>+'1'!K21+'2'!K21+'3'!K21+'4'!K21+'5'!K21+'6'!K21+'7'!K21+'8'!K21+'9'!K21+'10'!K21+'11'!K21+'12'!K21+'13'!K21+'14'!K21+'15'!K21+'16'!K21+'17'!K21+'18'!K21+'19'!K21+'20'!K21+'21'!K21+'22'!K21+'23'!K21+'24'!K21+'25'!K21+'26'!K21+'27'!K21+'28'!K21+'29'!K21+'30'!K21</f>
-        <v>0</v>
+        <v>50.848000000000006</v>
       </c>
       <c r="L12" s="286">
         <f>+'1'!L21+'2'!L21+'3'!L21+'4'!L21+'5'!L21+'6'!L21+'7'!L21+'8'!L21+'9'!L21+'10'!L21+'11'!L21+'12'!L21+'13'!L21+'14'!L21+'15'!L21+'16'!L21+'17'!L21+'18'!L21+'19'!L21+'20'!L21+'21'!L21+'22'!L21+'23'!L21+'24'!L21+'25'!L21+'26'!L21+'27'!L21+'28'!L21+'29'!L21+'30'!L21</f>
@@ -54794,19 +54797,19 @@
       </c>
       <c r="M12" s="230">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>1285.7280000000001</v>
       </c>
       <c r="N12" s="286">
         <f>+'1'!N21+'2'!N21+'3'!N21+'4'!N21+'5'!N21+'6'!N21+'7'!N21+'8'!N21+'9'!N21+'10'!N21+'11'!N21+'12'!N21+'13'!N21+'14'!N21+'15'!N21+'16'!N21+'17'!N21+'18'!N21+'19'!N21+'20'!N21+'21'!N21+'22'!N21+'23'!N21+'24'!N21+'25'!N21+'26'!N21+'27'!N21+'28'!N21+'29'!N21+'30'!N21</f>
-        <v>0</v>
+        <v>274.57627118644069</v>
       </c>
       <c r="O12" s="286">
         <f>+'1'!O21+'2'!O21+'3'!O21+'4'!O21+'5'!O21+'6'!O21+'7'!O21+'8'!O21+'9'!O21+'10'!O21+'11'!O21+'12'!O21+'13'!O21+'14'!O21+'15'!O21+'16'!O21+'17'!O21+'18'!O21+'19'!O21+'20'!O21+'21'!O21+'22'!O21+'23'!O21+'24'!O21+'25'!O21+'26'!O21+'27'!O21+'28'!O21+'29'!O21+'30'!O21</f>
-        <v>0</v>
+        <v>7.8015213559322039</v>
       </c>
       <c r="P12" s="311">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1568.1057925423729</v>
       </c>
       <c r="Q12" s="213">
         <f>+'1'!Q21+'2'!Q21+'3'!Q21+'4'!Q21+'5'!Q21+'6'!Q21+'7'!Q21+'8'!Q21+'9'!Q21+'10'!Q21+'11'!Q21+'12'!Q21+'13'!Q21+'14'!Q21+'15'!Q21+'16'!Q21+'17'!Q21+'18'!Q21+'19'!Q21+'20'!Q21+'21'!Q21+'22'!Q21+'23'!Q21+'24'!Q21+'25'!Q21+'26'!Q21+'27'!Q21+'28'!Q21+'29'!Q21+'30'!Q21</f>
@@ -54821,7 +54824,7 @@
       </c>
       <c r="T12" s="301">
         <f>+'10'!P35</f>
-        <v>2184.9047487266948</v>
+        <v>3136.2115850847458</v>
       </c>
     </row>
     <row r="13" spans="1:20 16377:16378" ht="21.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -54854,39 +54857,39 @@
       </c>
       <c r="H13" s="309">
         <f>+'1'!H22+'2'!H22+'3'!H22+'4'!H22+'5'!H22+'6'!H22+'7'!H22+'8'!H22+'9'!H22+'10'!H22+'11'!H22+'12'!H22+'13'!H22+'14'!H22+'15'!H22+'16'!H22+'17'!H22+'18'!H22+'19'!H22+'20'!H22+'21'!H22+'22'!H22+'23'!H22+'24'!H22+'25'!H22+'26'!H22+'27'!H22+'28'!H22+'29'!H22+'30'!H22</f>
-        <v>147</v>
+        <v>127</v>
       </c>
       <c r="I13" s="236">
         <f t="shared" si="0"/>
-        <v>5766.81</v>
+        <v>4982.2100000000009</v>
       </c>
       <c r="J13" s="286">
         <f>+'1'!J22+'2'!J22+'3'!J22+'4'!J22+'5'!J22+'6'!J22+'7'!J22+'8'!J22+'9'!J22+'10'!J22+'11'!J22+'12'!J22+'13'!J22+'14'!J22+'15'!J22+'16'!J22+'17'!J22+'18'!J22+'19'!J22+'20'!J22+'21'!J22+'22'!J22+'23'!J22+'24'!J22+'25'!J22+'26'!J22+'27'!J22+'28'!J22+'29'!J22+'30'!J22</f>
-        <v>288.34050000000008</v>
+        <v>249.11050000000009</v>
       </c>
       <c r="K13" s="286">
         <f>+'1'!K22+'2'!K22+'3'!K22+'4'!K22+'5'!K22+'6'!K22+'7'!K22+'8'!K22+'9'!K22+'10'!K22+'11'!K22+'12'!K22+'13'!K22+'14'!K22+'15'!K22+'16'!K22+'17'!K22+'18'!K22+'19'!K22+'20'!K22+'21'!K22+'22'!K22+'23'!K22+'24'!K22+'25'!K22+'26'!K22+'27'!K22+'28'!K22+'29'!K22+'30'!K22</f>
-        <v>201.83835000000005</v>
+        <v>174.37735000000004</v>
       </c>
       <c r="L13" s="286">
         <f>+'1'!L22+'2'!L22+'3'!L22+'4'!L22+'5'!L22+'6'!L22+'7'!L22+'8'!L22+'9'!L22+'10'!L22+'11'!L22+'12'!L22+'13'!L22+'14'!L22+'15'!L22+'16'!L22+'17'!L22+'18'!L22+'19'!L22+'20'!L22+'21'!L22+'22'!L22+'23'!L22+'24'!L22+'25'!L22+'26'!L22+'27'!L22+'28'!L22+'29'!L22+'30'!L22</f>
-        <v>294.10730999999998</v>
+        <v>254.09270999999998</v>
       </c>
       <c r="M13" s="230">
         <f t="shared" si="1"/>
-        <v>4982.5238399999998</v>
+        <v>4304.6294400000006</v>
       </c>
       <c r="N13" s="286">
         <f>+'1'!N22+'2'!N22+'3'!N22+'4'!N22+'5'!N22+'6'!N22+'7'!N22+'8'!N22+'9'!N22+'10'!N22+'11'!N22+'12'!N22+'13'!N22+'14'!N22+'15'!N22+'16'!N22+'17'!N22+'18'!N22+'19'!N22+'20'!N22+'21'!N22+'22'!N22+'23'!N22+'24'!N22+'25'!N22+'26'!N22+'27'!N22+'28'!N22+'29'!N22+'30'!N22</f>
-        <v>1121.1864406779655</v>
+        <v>968.64406779660976</v>
       </c>
       <c r="O13" s="286">
         <f>+'1'!O22+'2'!O22+'3'!O22+'4'!O22+'5'!O22+'6'!O22+'7'!O22+'8'!O22+'9'!O22+'10'!O22+'11'!O22+'12'!O22+'13'!O22+'14'!O22+'15'!O22+'16'!O22+'17'!O22+'18'!O22+'19'!O22+'20'!O22+'21'!O22+'22'!O22+'23'!O22+'24'!O22+'25'!O22+'26'!O22+'27'!O22+'28'!O22+'29'!O22+'30'!O22</f>
-        <v>30.518551403389832</v>
+        <v>26.366367538983052</v>
       </c>
       <c r="P13" s="311">
         <f t="shared" si="2"/>
-        <v>6134.2288320813559</v>
+        <v>5299.6398753355934</v>
       </c>
       <c r="Q13" s="213">
         <f>+'1'!Q22+'2'!Q22+'3'!Q22+'4'!Q22+'5'!Q22+'6'!Q22+'7'!Q22+'8'!Q22+'9'!Q22+'10'!Q22+'11'!Q22+'12'!Q22+'13'!Q22+'14'!Q22+'15'!Q22+'16'!Q22+'17'!Q22+'18'!Q22+'19'!Q22+'20'!Q22+'21'!Q22+'22'!Q22+'23'!Q22+'24'!Q22+'25'!Q22+'26'!Q22+'27'!Q22+'28'!Q22+'29'!Q22+'30'!Q22</f>
@@ -55086,35 +55089,35 @@
       </c>
       <c r="I16" s="114">
         <f t="shared" si="3"/>
-        <v>13151.900000000001</v>
+        <v>14021.875</v>
       </c>
       <c r="J16" s="274">
         <f>SUM(J7:J15)</f>
-        <v>879.14769999999999</v>
+        <v>972.28370000000007</v>
       </c>
       <c r="K16" s="275">
         <f t="shared" si="3"/>
-        <v>460.31650000000002</v>
+        <v>490.76562500000006</v>
       </c>
       <c r="L16" s="276">
         <f t="shared" si="3"/>
-        <v>294.10730999999998</v>
+        <v>254.09270999999998</v>
       </c>
       <c r="M16" s="232">
         <f t="shared" si="3"/>
-        <v>11518.32849</v>
+        <v>12304.732964999999</v>
       </c>
       <c r="N16" s="233">
         <f>SUM(N7:N15)</f>
-        <v>2516.9491525423718</v>
+        <v>2677.1186440677957</v>
       </c>
       <c r="O16" s="101">
         <f>SUM(O7:O15)</f>
-        <v>70.176388212711871</v>
+        <v>74.909258045338987</v>
       </c>
       <c r="P16" s="113">
         <f>SUM(P7:P15)</f>
-        <v>14105.454030755085</v>
+        <v>15056.760867113135</v>
       </c>
       <c r="Q16" s="128">
         <f>SUM(Q7:Q15)</f>
@@ -55201,7 +55204,7 @@
       <c r="O19" s="366"/>
       <c r="P19" s="139">
         <f>I16</f>
-        <v>13151.900000000001</v>
+        <v>14021.875</v>
       </c>
       <c r="R19" s="299">
         <v>17</v>
@@ -55233,7 +55236,7 @@
       <c r="O20" s="368"/>
       <c r="P20" s="140">
         <f>+J16</f>
-        <v>879.14769999999999</v>
+        <v>972.28370000000007</v>
       </c>
       <c r="R20" s="299">
         <v>18</v>
@@ -55265,7 +55268,7 @@
       <c r="O21" s="368"/>
       <c r="P21" s="140">
         <f>+K16+L16</f>
-        <v>754.42381</v>
+        <v>744.85833500000001</v>
       </c>
       <c r="R21" s="299">
         <v>19</v>
@@ -55298,7 +55301,7 @@
       <c r="O22" s="368"/>
       <c r="P22" s="140">
         <f>P19-P20-P21</f>
-        <v>11518.328490000002</v>
+        <v>12304.732964999999</v>
       </c>
       <c r="R22" s="299">
         <v>20</v>
@@ -55333,7 +55336,7 @@
       </c>
       <c r="P23" s="140">
         <f>+N16</f>
-        <v>2516.9491525423718</v>
+        <v>2677.1186440677957</v>
       </c>
       <c r="R23" s="299">
         <v>21</v>
@@ -55366,7 +55369,7 @@
       <c r="O24" s="370"/>
       <c r="P24" s="140">
         <f>P22+P23</f>
-        <v>14035.277642542373</v>
+        <v>14981.851609067795</v>
       </c>
       <c r="R24" s="299">
         <v>22</v>
@@ -55402,7 +55405,7 @@
       </c>
       <c r="P25" s="140">
         <f>+O16</f>
-        <v>70.176388212711871</v>
+        <v>74.909258045338987</v>
       </c>
       <c r="R25" s="299">
         <v>23</v>
@@ -55423,7 +55426,7 @@
       <c r="O26" s="372"/>
       <c r="P26" s="297">
         <f>+P24+P25</f>
-        <v>14105.454030755085</v>
+        <v>15056.760867113135</v>
       </c>
       <c r="R26" s="299">
         <v>24</v>
@@ -55537,7 +55540,7 @@
       </c>
       <c r="T33" s="304">
         <f>SUM(T3:T32)</f>
-        <v>14105.454030755081</v>
+        <v>15056.760867113133</v>
       </c>
     </row>
     <row r="44" spans="2:20" x14ac:dyDescent="0.35">

</xml_diff>